<commit_message>
Update infrastructure costing spreadsheet with detailed formatting
Regenerate the infrastructure costing spreadsheet (attached_assets/CuraLive_Infrastructure_Costs_Updated.xlsx) to precisely match the original file's formatting, including specific number formats, cell colors, borders, and header styles.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 0cbe7a84-a7a6-4a51-b09c-2be09cbda9ee
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 3c326660-0fc0-4de7-9fd3-f79873321e2b
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/1f99a8d9-3543-48bc-8564-b0463564e29d/0cbe7a84-a7a6-4a51-b09c-2be09cbda9ee/DdXNYUA
</commit_message>
<xml_diff>
--- a/attached_assets/CuraLive_Infrastructure_Costs_Updated.xlsx
+++ b/attached_assets/CuraLive_Infrastructure_Costs_Updated.xlsx
@@ -351,7 +351,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="7" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+  </numFmts>
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -361,41 +364,41 @@
     </font>
     <font>
       <b/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FFe2e8f0"/>
+      <sz val="11"/>
+    </font>
+    <font>
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <color rgb="FF333333"/>
-      <sz val="10"/>
-      <name val="Calibri"/>
+      <b/>
+      <color rgb="FF34d399"/>
+      <sz val="11"/>
     </font>
     <font>
-      <i/>
-      <color rgb="FF666666"/>
-      <sz val="10"/>
+      <b/>
+      <sz val="11"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <color rgb="FF1B5E20"/>
-      <sz val="10"/>
-      <name val="Calibri"/>
+      <color rgb="FF34d399"/>
+      <sz val="14"/>
     </font>
     <font>
       <b/>
-      <color rgb="FF4ADE80"/>
-      <sz val="14"/>
-      <name val="Calibri"/>
+      <color rgb="FFe2e8f0"/>
+      <sz val="12"/>
     </font>
     <font>
-      <b/>
-      <color rgb="FF333333"/>
+      <i/>
+      <color rgb="FF94a3b8"/>
       <sz val="10"/>
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -404,12 +407,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1A1F2E"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF8F8F8"/>
+        <fgColor rgb="FF1a1f2e"/>
       </patternFill>
     </fill>
     <fill>
@@ -419,7 +417,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFE8F5E9"/>
+        <fgColor rgb="FF0f3d1e"/>
       </patternFill>
     </fill>
     <fill>
@@ -443,31 +441,25 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FF3A3F4E"/>
+        <color rgb="FF334155"/>
       </left>
       <right style="thin">
-        <color rgb="FF3A3F4E"/>
+        <color rgb="FF334155"/>
       </right>
       <top style="thin">
-        <color rgb="FF3A3F4E"/>
+        <color rgb="FF334155"/>
       </top>
       <bottom style="thin">
-        <color rgb="FF3A3F4E"/>
+        <color rgb="FF334155"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FFE0E0E0"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFE0E0E0"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFE0E0E0"/>
-      </top>
+      <left/>
+      <right/>
+      <top/>
       <bottom style="thin">
-        <color rgb="FFE0E0E0"/>
+        <color rgb="FF1e293b"/>
       </bottom>
       <diagonal/>
     </border>
@@ -478,38 +470,42 @@
   <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -849,9 +845,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr>
-    <tabColor rgb="1A1F2E"/>
-  </sheetPr>
   <dimension ref="A1:I23"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
@@ -866,7 +859,7 @@
     <col min="9" max="9" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -895,236 +888,236 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
+      <c r="F2" s="3"/>
       <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-    </row>
-    <row r="3" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
       <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
+      <c r="G3" s="2"/>
       <c r="H3" s="3"/>
       <c r="I3" s="3"/>
     </row>
-    <row r="4" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
+      <c r="F4" s="3"/>
       <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
-    </row>
-    <row r="5" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" s="2"/>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
       <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
+      <c r="G5" s="2"/>
       <c r="H5" s="3"/>
       <c r="I5" s="3"/>
     </row>
-    <row r="6" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
+      <c r="F6" s="3"/>
       <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
-      <c r="I6" s="2"/>
-    </row>
-    <row r="7" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="3"/>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" s="2"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
       <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
+      <c r="G7" s="2"/>
       <c r="H7" s="3"/>
       <c r="I7" s="3"/>
     </row>
-    <row r="8" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
+      <c r="F8" s="3"/>
       <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
-      <c r="I8" s="2"/>
-    </row>
-    <row r="9" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="3"/>
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" s="2"/>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2"/>
       <c r="F9" s="3"/>
-      <c r="G9" s="3"/>
+      <c r="G9" s="2"/>
       <c r="H9" s="3"/>
       <c r="I9" s="3"/>
     </row>
-    <row r="10" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
+      <c r="F10" s="3"/>
       <c r="G10" s="2"/>
-      <c r="H10" s="2"/>
-      <c r="I10" s="2"/>
-    </row>
-    <row r="11" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" s="3"/>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
+      <c r="H10" s="3"/>
+      <c r="I10" s="3"/>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" s="2"/>
+      <c r="B11" s="2"/>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2"/>
       <c r="F11" s="3"/>
-      <c r="G11" s="3"/>
+      <c r="G11" s="2"/>
       <c r="H11" s="3"/>
       <c r="I11" s="3"/>
     </row>
-    <row r="12" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
+      <c r="F12" s="3"/>
       <c r="G12" s="2"/>
-      <c r="H12" s="2"/>
-      <c r="I12" s="2"/>
-    </row>
-    <row r="13" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" s="3"/>
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3"/>
+      <c r="H12" s="3"/>
+      <c r="I12" s="3"/>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" s="2"/>
+      <c r="B13" s="2"/>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2"/>
       <c r="F13" s="3"/>
-      <c r="G13" s="3"/>
+      <c r="G13" s="2"/>
       <c r="H13" s="3"/>
       <c r="I13" s="3"/>
     </row>
-    <row r="14" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
+      <c r="F14" s="3"/>
       <c r="G14" s="2"/>
-      <c r="H14" s="2"/>
-      <c r="I14" s="2"/>
-    </row>
-    <row r="15" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A15" s="3"/>
-      <c r="B15" s="3"/>
-      <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
-      <c r="E15" s="3"/>
+      <c r="H14" s="3"/>
+      <c r="I14" s="3"/>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" s="2"/>
+      <c r="B15" s="2"/>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2"/>
       <c r="F15" s="3"/>
-      <c r="G15" s="3"/>
+      <c r="G15" s="2"/>
       <c r="H15" s="3"/>
       <c r="I15" s="3"/>
     </row>
-    <row r="16" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
+      <c r="F16" s="3"/>
       <c r="G16" s="2"/>
-      <c r="H16" s="2"/>
-      <c r="I16" s="2"/>
-    </row>
-    <row r="17" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A17" s="3"/>
-      <c r="B17" s="3"/>
-      <c r="C17" s="3"/>
-      <c r="D17" s="3"/>
-      <c r="E17" s="3"/>
+      <c r="H16" s="3"/>
+      <c r="I16" s="3"/>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A17" s="2"/>
+      <c r="B17" s="2"/>
+      <c r="C17" s="2"/>
+      <c r="D17" s="2"/>
+      <c r="E17" s="2"/>
       <c r="F17" s="3"/>
-      <c r="G17" s="3"/>
+      <c r="G17" s="2"/>
       <c r="H17" s="3"/>
       <c r="I17" s="3"/>
     </row>
-    <row r="18" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="2"/>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
       <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
+      <c r="F18" s="3"/>
       <c r="G18" s="2"/>
-      <c r="H18" s="2"/>
-      <c r="I18" s="2"/>
-    </row>
-    <row r="19" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A19" s="3"/>
-      <c r="B19" s="3"/>
-      <c r="C19" s="3"/>
-      <c r="D19" s="3"/>
-      <c r="E19" s="3"/>
+      <c r="H18" s="3"/>
+      <c r="I18" s="3"/>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19" s="2"/>
+      <c r="B19" s="2"/>
+      <c r="C19" s="2"/>
+      <c r="D19" s="2"/>
+      <c r="E19" s="2"/>
       <c r="F19" s="3"/>
-      <c r="G19" s="3"/>
+      <c r="G19" s="2"/>
       <c r="H19" s="3"/>
       <c r="I19" s="3"/>
     </row>
-    <row r="20" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="2"/>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
       <c r="E20" s="2"/>
-      <c r="F20" s="2"/>
+      <c r="F20" s="3"/>
       <c r="G20" s="2"/>
-      <c r="H20" s="2"/>
-      <c r="I20" s="2"/>
-    </row>
-    <row r="21" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A21" s="3"/>
-      <c r="B21" s="3"/>
-      <c r="C21" s="3"/>
-      <c r="D21" s="3"/>
-      <c r="E21" s="3"/>
+      <c r="H20" s="3"/>
+      <c r="I20" s="3"/>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21" s="2"/>
+      <c r="B21" s="2"/>
+      <c r="C21" s="2"/>
+      <c r="D21" s="2"/>
+      <c r="E21" s="2"/>
       <c r="F21" s="3"/>
-      <c r="G21" s="3"/>
+      <c r="G21" s="2"/>
       <c r="H21" s="3"/>
       <c r="I21" s="3"/>
     </row>
-    <row r="22" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
       <c r="D22" s="2"/>
       <c r="E22" s="2"/>
-      <c r="F22" s="2"/>
+      <c r="F22" s="3"/>
       <c r="G22" s="2"/>
-      <c r="H22" s="2"/>
-      <c r="I22" s="2"/>
+      <c r="H22" s="3"/>
+      <c r="I22" s="3"/>
     </row>
     <row r="23" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="4"/>
@@ -1132,9 +1125,9 @@
       <c r="C23" s="4"/>
       <c r="D23" s="4"/>
       <c r="E23" s="4"/>
-      <c r="F23" s="4"/>
+      <c r="F23" s="5"/>
       <c r="G23" s="4"/>
-      <c r="H23" s="4"/>
+      <c r="H23" s="5"/>
       <c r="I23" s="4"/>
     </row>
   </sheetData>
@@ -1145,21 +1138,19 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr>
-    <tabColor rgb="1A1F2E"/>
-  </sheetPr>
   <dimension ref="A1:L14"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="22" customWidth="1"/>
     <col min="3" max="5" width="24" customWidth="1"/>
     <col min="6" max="6" width="50" customWidth="1"/>
-    <col min="7" max="10" width="18" customWidth="1"/>
+    <col min="7" max="9" width="20" customWidth="1"/>
+    <col min="10" max="10" width="18" customWidth="1"/>
     <col min="11" max="11" width="16" customWidth="1"/>
-    <col min="12" max="12" width="20" customWidth="1"/>
+    <col min="12" max="12" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" ht="22" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>9</v>
       </c>
@@ -1197,27 +1188,27 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" ht="22" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
-      <c r="K2" s="2"/>
-      <c r="L2" s="2"/>
-    </row>
-    <row r="3" ht="22" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3"/>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
       <c r="G3" s="3"/>
       <c r="H3" s="3"/>
       <c r="I3" s="3"/>
@@ -1225,27 +1216,27 @@
       <c r="K3" s="3"/>
       <c r="L3" s="3"/>
     </row>
-    <row r="4" ht="22" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
-      <c r="J4" s="2"/>
-      <c r="K4" s="2"/>
-      <c r="L4" s="2"/>
-    </row>
-    <row r="5" ht="22" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
+      <c r="L4" s="3"/>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A5" s="2"/>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
       <c r="G5" s="3"/>
       <c r="H5" s="3"/>
       <c r="I5" s="3"/>
@@ -1253,133 +1244,133 @@
       <c r="K5" s="3"/>
       <c r="L5" s="3"/>
     </row>
-    <row r="7" ht="28" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
+    <row r="7" ht="26" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A7" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="B7" s="4"/>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4"/>
-      <c r="G7" s="4"/>
-      <c r="H7" s="4"/>
-      <c r="I7" s="4"/>
-      <c r="J7" s="4"/>
-      <c r="K7" s="4"/>
-      <c r="L7" s="4"/>
-    </row>
-    <row r="8" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A8" s="5" t="s">
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
+      <c r="J7" s="6"/>
+      <c r="K7" s="6"/>
+      <c r="L7" s="6"/>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A8" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="B8" s="5"/>
-      <c r="C8" s="5"/>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
-      <c r="F8" s="5"/>
-      <c r="G8" s="5"/>
-      <c r="H8" s="5"/>
-      <c r="I8" s="5"/>
-      <c r="J8" s="5"/>
-      <c r="K8" s="5"/>
-      <c r="L8" s="5"/>
-    </row>
-    <row r="9" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A9" s="5" t="s">
+      <c r="B8" s="7"/>
+      <c r="C8" s="7"/>
+      <c r="D8" s="7"/>
+      <c r="E8" s="7"/>
+      <c r="F8" s="7"/>
+      <c r="G8" s="7"/>
+      <c r="H8" s="7"/>
+      <c r="I8" s="7"/>
+      <c r="J8" s="7"/>
+      <c r="K8" s="7"/>
+      <c r="L8" s="7"/>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A9" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="B9" s="5"/>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
-      <c r="F9" s="5"/>
-      <c r="G9" s="5"/>
-      <c r="H9" s="5"/>
-      <c r="I9" s="5"/>
-      <c r="J9" s="5"/>
-      <c r="K9" s="5"/>
-      <c r="L9" s="5"/>
-    </row>
-    <row r="10" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A10" s="5" t="s">
+      <c r="B9" s="7"/>
+      <c r="C9" s="7"/>
+      <c r="D9" s="7"/>
+      <c r="E9" s="7"/>
+      <c r="F9" s="7"/>
+      <c r="G9" s="7"/>
+      <c r="H9" s="7"/>
+      <c r="I9" s="7"/>
+      <c r="J9" s="7"/>
+      <c r="K9" s="7"/>
+      <c r="L9" s="7"/>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A10" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="B10" s="5"/>
-      <c r="C10" s="5"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-      <c r="F10" s="5"/>
-      <c r="G10" s="5"/>
-      <c r="H10" s="5"/>
-      <c r="I10" s="5"/>
-      <c r="J10" s="5"/>
-      <c r="K10" s="5"/>
-      <c r="L10" s="5"/>
-    </row>
-    <row r="11" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A11" s="5" t="s">
+      <c r="B10" s="7"/>
+      <c r="C10" s="7"/>
+      <c r="D10" s="7"/>
+      <c r="E10" s="7"/>
+      <c r="F10" s="7"/>
+      <c r="G10" s="7"/>
+      <c r="H10" s="7"/>
+      <c r="I10" s="7"/>
+      <c r="J10" s="7"/>
+      <c r="K10" s="7"/>
+      <c r="L10" s="7"/>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A11" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="B11" s="5"/>
-      <c r="C11" s="5"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
-      <c r="F11" s="5"/>
-      <c r="G11" s="5"/>
-      <c r="H11" s="5"/>
-      <c r="I11" s="5"/>
-      <c r="J11" s="5"/>
-      <c r="K11" s="5"/>
-      <c r="L11" s="5"/>
-    </row>
-    <row r="12" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A12" s="5" t="s">
+      <c r="B11" s="7"/>
+      <c r="C11" s="7"/>
+      <c r="D11" s="7"/>
+      <c r="E11" s="7"/>
+      <c r="F11" s="7"/>
+      <c r="G11" s="7"/>
+      <c r="H11" s="7"/>
+      <c r="I11" s="7"/>
+      <c r="J11" s="7"/>
+      <c r="K11" s="7"/>
+      <c r="L11" s="7"/>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A12" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B12" s="5"/>
-      <c r="C12" s="5"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
-      <c r="F12" s="5"/>
-      <c r="G12" s="5"/>
-      <c r="H12" s="5"/>
-      <c r="I12" s="5"/>
-      <c r="J12" s="5"/>
-      <c r="K12" s="5"/>
-      <c r="L12" s="5"/>
-    </row>
-    <row r="13" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A13" s="5" t="s">
+      <c r="B12" s="7"/>
+      <c r="C12" s="7"/>
+      <c r="D12" s="7"/>
+      <c r="E12" s="7"/>
+      <c r="F12" s="7"/>
+      <c r="G12" s="7"/>
+      <c r="H12" s="7"/>
+      <c r="I12" s="7"/>
+      <c r="J12" s="7"/>
+      <c r="K12" s="7"/>
+      <c r="L12" s="7"/>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A13" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="B13" s="5"/>
-      <c r="C13" s="5"/>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
-      <c r="F13" s="5"/>
-      <c r="G13" s="5"/>
-      <c r="H13" s="5"/>
-      <c r="I13" s="5"/>
-      <c r="J13" s="5"/>
-      <c r="K13" s="5"/>
-      <c r="L13" s="5"/>
-    </row>
-    <row r="14" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A14" s="5" t="s">
+      <c r="B13" s="7"/>
+      <c r="C13" s="7"/>
+      <c r="D13" s="7"/>
+      <c r="E13" s="7"/>
+      <c r="F13" s="7"/>
+      <c r="G13" s="7"/>
+      <c r="H13" s="7"/>
+      <c r="I13" s="7"/>
+      <c r="J13" s="7"/>
+      <c r="K13" s="7"/>
+      <c r="L13" s="7"/>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A14" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="B14" s="5"/>
-      <c r="C14" s="5"/>
-      <c r="D14" s="5"/>
-      <c r="E14" s="5"/>
-      <c r="F14" s="5"/>
-      <c r="G14" s="5"/>
-      <c r="H14" s="5"/>
-      <c r="I14" s="5"/>
-      <c r="J14" s="5"/>
-      <c r="K14" s="5"/>
-      <c r="L14" s="5"/>
+      <c r="B14" s="7"/>
+      <c r="C14" s="7"/>
+      <c r="D14" s="7"/>
+      <c r="E14" s="7"/>
+      <c r="F14" s="7"/>
+      <c r="G14" s="7"/>
+      <c r="H14" s="7"/>
+      <c r="I14" s="7"/>
+      <c r="J14" s="7"/>
+      <c r="K14" s="7"/>
+      <c r="L14" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -1399,16 +1390,14 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr>
-    <tabColor rgb="1A1F2E"/>
-  </sheetPr>
   <dimension ref="A1:K18"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
     <col min="3" max="3" width="55" customWidth="1"/>
-    <col min="4" max="6" width="16" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="6" width="16" customWidth="1"/>
     <col min="7" max="7" width="14" customWidth="1"/>
     <col min="8" max="8" width="12" customWidth="1"/>
     <col min="9" max="9" width="10" customWidth="1"/>
@@ -1416,7 +1405,7 @@
     <col min="11" max="11" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" ht="22" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>29</v>
       </c>
@@ -1451,23 +1440,23 @@
         <v>38</v>
       </c>
     </row>
-    <row r="2" ht="22" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
-      <c r="K2" s="2"/>
-    </row>
-    <row r="3" ht="22" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3"/>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
       <c r="D3" s="3"/>
       <c r="E3" s="3"/>
       <c r="F3" s="3"/>
@@ -1477,23 +1466,23 @@
       <c r="J3" s="3"/>
       <c r="K3" s="3"/>
     </row>
-    <row r="4" ht="22" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
-      <c r="J4" s="2"/>
-      <c r="K4" s="2"/>
-    </row>
-    <row r="5" ht="22" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" s="2"/>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
       <c r="D5" s="3"/>
       <c r="E5" s="3"/>
       <c r="F5" s="3"/>
@@ -1503,23 +1492,23 @@
       <c r="J5" s="3"/>
       <c r="K5" s="3"/>
     </row>
-    <row r="6" ht="22" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" s="6"/>
-      <c r="B6" s="6"/>
-      <c r="C6" s="6"/>
-      <c r="D6" s="6"/>
-      <c r="E6" s="6"/>
-      <c r="F6" s="6"/>
-      <c r="G6" s="6"/>
-      <c r="H6" s="6"/>
-      <c r="I6" s="6"/>
-      <c r="J6" s="6"/>
-      <c r="K6" s="6"/>
-    </row>
-    <row r="7" ht="22" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" s="3"/>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" s="8"/>
+      <c r="B6" s="8"/>
+      <c r="C6" s="8"/>
+      <c r="D6" s="9"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="9"/>
+      <c r="G6" s="9"/>
+      <c r="H6" s="9"/>
+      <c r="I6" s="9"/>
+      <c r="J6" s="9"/>
+      <c r="K6" s="9"/>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" s="2"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
       <c r="D7" s="3"/>
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
@@ -1529,23 +1518,23 @@
       <c r="J7" s="3"/>
       <c r="K7" s="3"/>
     </row>
-    <row r="8" ht="22" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
-      <c r="I8" s="2"/>
-      <c r="J8" s="2"/>
-      <c r="K8" s="2"/>
-    </row>
-    <row r="9" ht="22" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A9" s="3"/>
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
+      <c r="J8" s="3"/>
+      <c r="K8" s="3"/>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9" s="2"/>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
       <c r="F9" s="3"/>
@@ -1555,23 +1544,23 @@
       <c r="J9" s="3"/>
       <c r="K9" s="3"/>
     </row>
-    <row r="10" ht="22" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
-      <c r="H10" s="2"/>
-      <c r="I10" s="2"/>
-      <c r="J10" s="2"/>
-      <c r="K10" s="2"/>
-    </row>
-    <row r="11" ht="22" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A11" s="3"/>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+      <c r="I10" s="3"/>
+      <c r="J10" s="3"/>
+      <c r="K10" s="3"/>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A11" s="2"/>
+      <c r="B11" s="2"/>
+      <c r="C11" s="2"/>
       <c r="D11" s="3"/>
       <c r="E11" s="3"/>
       <c r="F11" s="3"/>
@@ -1581,95 +1570,95 @@
       <c r="J11" s="3"/>
       <c r="K11" s="3"/>
     </row>
-    <row r="13" ht="28" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A13" s="7" t="s">
+    <row r="13" ht="26" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A13" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="B13" s="7"/>
-      <c r="C13" s="7"/>
-      <c r="D13" s="7"/>
-      <c r="E13" s="7"/>
-      <c r="F13" s="7"/>
-      <c r="G13" s="7"/>
-      <c r="H13" s="7"/>
-      <c r="I13" s="7"/>
-      <c r="J13" s="7"/>
-      <c r="K13" s="7"/>
-    </row>
-    <row r="14" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A14" s="5" t="s">
+      <c r="B13" s="10"/>
+      <c r="C13" s="10"/>
+      <c r="D13" s="10"/>
+      <c r="E13" s="10"/>
+      <c r="F13" s="10"/>
+      <c r="G13" s="10"/>
+      <c r="H13" s="10"/>
+      <c r="I13" s="10"/>
+      <c r="J13" s="10"/>
+      <c r="K13" s="10"/>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A14" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="B14" s="5"/>
-      <c r="C14" s="5"/>
-      <c r="D14" s="5"/>
-      <c r="E14" s="5"/>
-      <c r="F14" s="5"/>
-      <c r="G14" s="5"/>
-      <c r="H14" s="5"/>
-      <c r="I14" s="5"/>
-      <c r="J14" s="5"/>
-      <c r="K14" s="5"/>
-    </row>
-    <row r="15" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A15" s="5" t="s">
+      <c r="B14" s="7"/>
+      <c r="C14" s="7"/>
+      <c r="D14" s="7"/>
+      <c r="E14" s="7"/>
+      <c r="F14" s="7"/>
+      <c r="G14" s="7"/>
+      <c r="H14" s="7"/>
+      <c r="I14" s="7"/>
+      <c r="J14" s="7"/>
+      <c r="K14" s="7"/>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A15" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="B15" s="5"/>
-      <c r="C15" s="5"/>
-      <c r="D15" s="5"/>
-      <c r="E15" s="5"/>
-      <c r="F15" s="5"/>
-      <c r="G15" s="5"/>
-      <c r="H15" s="5"/>
-      <c r="I15" s="5"/>
-      <c r="J15" s="5"/>
-      <c r="K15" s="5"/>
-    </row>
-    <row r="16" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A16" s="5" t="s">
+      <c r="B15" s="7"/>
+      <c r="C15" s="7"/>
+      <c r="D15" s="7"/>
+      <c r="E15" s="7"/>
+      <c r="F15" s="7"/>
+      <c r="G15" s="7"/>
+      <c r="H15" s="7"/>
+      <c r="I15" s="7"/>
+      <c r="J15" s="7"/>
+      <c r="K15" s="7"/>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A16" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="B16" s="5"/>
-      <c r="C16" s="5"/>
-      <c r="D16" s="5"/>
-      <c r="E16" s="5"/>
-      <c r="F16" s="5"/>
-      <c r="G16" s="5"/>
-      <c r="H16" s="5"/>
-      <c r="I16" s="5"/>
-      <c r="J16" s="5"/>
-      <c r="K16" s="5"/>
-    </row>
-    <row r="17" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A17" s="5" t="s">
+      <c r="B16" s="7"/>
+      <c r="C16" s="7"/>
+      <c r="D16" s="7"/>
+      <c r="E16" s="7"/>
+      <c r="F16" s="7"/>
+      <c r="G16" s="7"/>
+      <c r="H16" s="7"/>
+      <c r="I16" s="7"/>
+      <c r="J16" s="7"/>
+      <c r="K16" s="7"/>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A17" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B17" s="5"/>
-      <c r="C17" s="5"/>
-      <c r="D17" s="5"/>
-      <c r="E17" s="5"/>
-      <c r="F17" s="5"/>
-      <c r="G17" s="5"/>
-      <c r="H17" s="5"/>
-      <c r="I17" s="5"/>
-      <c r="J17" s="5"/>
-      <c r="K17" s="5"/>
-    </row>
-    <row r="18" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A18" s="5" t="s">
+      <c r="B17" s="7"/>
+      <c r="C17" s="7"/>
+      <c r="D17" s="7"/>
+      <c r="E17" s="7"/>
+      <c r="F17" s="7"/>
+      <c r="G17" s="7"/>
+      <c r="H17" s="7"/>
+      <c r="I17" s="7"/>
+      <c r="J17" s="7"/>
+      <c r="K17" s="7"/>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A18" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="B18" s="5"/>
-      <c r="C18" s="5"/>
-      <c r="D18" s="5"/>
-      <c r="E18" s="5"/>
-      <c r="F18" s="5"/>
-      <c r="G18" s="5"/>
-      <c r="H18" s="5"/>
-      <c r="I18" s="5"/>
-      <c r="J18" s="5"/>
-      <c r="K18" s="5"/>
+      <c r="B18" s="7"/>
+      <c r="C18" s="7"/>
+      <c r="D18" s="7"/>
+      <c r="E18" s="7"/>
+      <c r="F18" s="7"/>
+      <c r="G18" s="7"/>
+      <c r="H18" s="7"/>
+      <c r="I18" s="7"/>
+      <c r="J18" s="7"/>
+      <c r="K18" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -1687,13 +1676,10 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr>
-    <tabColor rgb="1A1F2E"/>
-  </sheetPr>
   <dimension ref="A1:O13"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="22" customWidth="1"/>
+    <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="3" width="16" customWidth="1"/>
     <col min="4" max="5" width="14" customWidth="1"/>
     <col min="6" max="6" width="16" customWidth="1"/>
@@ -1704,7 +1690,7 @@
     <col min="15" max="15" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" ht="22" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>45</v>
       </c>
@@ -1751,7 +1737,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="2" ht="22" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1760,32 +1746,32 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
-      <c r="K2" s="2"/>
-      <c r="L2" s="2"/>
-      <c r="M2" s="2"/>
-      <c r="N2" s="2"/>
-      <c r="O2" s="2"/>
-    </row>
-    <row r="3" ht="22" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A3" s="6"/>
-      <c r="B3" s="6"/>
-      <c r="C3" s="6"/>
-      <c r="D3" s="6"/>
-      <c r="E3" s="6"/>
-      <c r="F3" s="6"/>
-      <c r="G3" s="6"/>
-      <c r="H3" s="6"/>
-      <c r="I3" s="6"/>
-      <c r="J3" s="6"/>
-      <c r="K3" s="6"/>
-      <c r="L3" s="6"/>
-      <c r="M3" s="6"/>
-      <c r="N3" s="6"/>
-      <c r="O3" s="6"/>
-    </row>
-    <row r="4" ht="22" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3"/>
+      <c r="M2" s="3"/>
+      <c r="N2" s="3"/>
+      <c r="O2" s="3"/>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A3" s="8"/>
+      <c r="B3" s="8"/>
+      <c r="C3" s="8"/>
+      <c r="D3" s="8"/>
+      <c r="E3" s="8"/>
+      <c r="F3" s="8"/>
+      <c r="G3" s="8"/>
+      <c r="H3" s="8"/>
+      <c r="I3" s="9"/>
+      <c r="J3" s="9"/>
+      <c r="K3" s="9"/>
+      <c r="L3" s="9"/>
+      <c r="M3" s="9"/>
+      <c r="N3" s="9"/>
+      <c r="O3" s="9"/>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -1794,23 +1780,23 @@
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
       <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
-      <c r="J4" s="2"/>
-      <c r="K4" s="2"/>
-      <c r="L4" s="2"/>
-      <c r="M4" s="2"/>
-      <c r="N4" s="2"/>
-      <c r="O4" s="2"/>
-    </row>
-    <row r="5" ht="22" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
-      <c r="H5" s="3"/>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
+      <c r="L4" s="3"/>
+      <c r="M4" s="3"/>
+      <c r="N4" s="3"/>
+      <c r="O4" s="3"/>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A5" s="2"/>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
+      <c r="H5" s="2"/>
       <c r="I5" s="3"/>
       <c r="J5" s="3"/>
       <c r="K5" s="3"/>
@@ -1819,7 +1805,7 @@
       <c r="N5" s="3"/>
       <c r="O5" s="3"/>
     </row>
-    <row r="6" ht="22" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
@@ -1828,23 +1814,23 @@
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
-      <c r="I6" s="2"/>
-      <c r="J6" s="2"/>
-      <c r="K6" s="2"/>
-      <c r="L6" s="2"/>
-      <c r="M6" s="2"/>
-      <c r="N6" s="2"/>
-      <c r="O6" s="2"/>
-    </row>
-    <row r="7" ht="22" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A7" s="3"/>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
-      <c r="H7" s="3"/>
+      <c r="I6" s="3"/>
+      <c r="J6" s="3"/>
+      <c r="K6" s="3"/>
+      <c r="L6" s="3"/>
+      <c r="M6" s="3"/>
+      <c r="N6" s="3"/>
+      <c r="O6" s="3"/>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A7" s="2"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
       <c r="I7" s="3"/>
       <c r="J7" s="3"/>
       <c r="K7" s="3"/>
@@ -1853,26 +1839,26 @@
       <c r="N7" s="3"/>
       <c r="O7" s="3"/>
     </row>
-    <row r="9" ht="28" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A9" s="8" t="s">
+    <row r="9" ht="26" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A9" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="B9" s="8"/>
-      <c r="C9" s="8"/>
-      <c r="D9" s="8"/>
-      <c r="E9" s="8"/>
-      <c r="F9" s="8"/>
-      <c r="G9" s="8"/>
-      <c r="H9" s="8"/>
-      <c r="I9" s="8"/>
-      <c r="J9" s="8"/>
-      <c r="K9" s="8"/>
-      <c r="L9" s="8"/>
-      <c r="M9" s="8"/>
-      <c r="N9" s="8"/>
-      <c r="O9" s="8"/>
-    </row>
-    <row r="10" ht="22" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="B9" s="11"/>
+      <c r="C9" s="11"/>
+      <c r="D9" s="11"/>
+      <c r="E9" s="11"/>
+      <c r="F9" s="11"/>
+      <c r="G9" s="11"/>
+      <c r="H9" s="11"/>
+      <c r="I9" s="11"/>
+      <c r="J9" s="11"/>
+      <c r="K9" s="11"/>
+      <c r="L9" s="11"/>
+      <c r="M9" s="11"/>
+      <c r="N9" s="11"/>
+      <c r="O9" s="11"/>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -1881,30 +1867,30 @@
       <c r="F10" s="2"/>
       <c r="G10" s="2"/>
       <c r="H10" s="2"/>
-      <c r="I10" s="2"/>
-      <c r="J10" s="2"/>
-      <c r="K10" s="2"/>
-      <c r="L10" s="2"/>
-      <c r="M10" s="2"/>
-      <c r="N10" s="2"/>
-      <c r="O10" s="2"/>
-    </row>
-    <row r="11" ht="22" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A11" s="3"/>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
-      <c r="F11" s="3"/>
-      <c r="G11" s="3"/>
-      <c r="H11" s="3"/>
-      <c r="I11" s="3"/>
-      <c r="J11" s="3"/>
-      <c r="K11" s="3"/>
-      <c r="L11" s="3"/>
-      <c r="M11" s="3"/>
-      <c r="N11" s="3"/>
-      <c r="O11" s="3"/>
+      <c r="I10" s="3"/>
+      <c r="J10" s="3"/>
+      <c r="K10" s="3"/>
+      <c r="L10" s="3"/>
+      <c r="M10" s="3"/>
+      <c r="N10" s="3"/>
+      <c r="O10" s="3"/>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A11" s="8"/>
+      <c r="B11" s="8"/>
+      <c r="C11" s="8"/>
+      <c r="D11" s="8"/>
+      <c r="E11" s="8"/>
+      <c r="F11" s="8"/>
+      <c r="G11" s="8"/>
+      <c r="H11" s="8"/>
+      <c r="I11" s="9"/>
+      <c r="J11" s="9"/>
+      <c r="K11" s="9"/>
+      <c r="L11" s="9"/>
+      <c r="M11" s="9"/>
+      <c r="N11" s="9"/>
+      <c r="O11" s="9"/>
     </row>
     <row r="12" ht="26" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="4"/>
@@ -1917,14 +1903,14 @@
       <c r="H12" s="4"/>
       <c r="I12" s="4"/>
       <c r="J12" s="4"/>
-      <c r="K12" s="4"/>
+      <c r="K12" s="5"/>
       <c r="L12" s="4"/>
-      <c r="M12" s="4"/>
+      <c r="M12" s="5"/>
       <c r="N12" s="4"/>
-      <c r="O12" s="4"/>
+      <c r="O12" s="5"/>
     </row>
     <row r="13" spans="15:15" x14ac:dyDescent="0.25">
-      <c r="O13" s="9"/>
+      <c r="O13" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1937,9 +1923,6 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr>
-    <tabColor rgb="1A1F2E"/>
-  </sheetPr>
   <dimension ref="A1:K15"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
@@ -1951,7 +1934,7 @@
     <col min="11" max="11" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" ht="22" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>60</v>
       </c>
@@ -1986,186 +1969,186 @@
         <v>70</v>
       </c>
     </row>
-    <row r="2" ht="22" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
-      <c r="K2" s="2"/>
-    </row>
-    <row r="3" ht="22" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3"/>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" s="2"/>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
       <c r="H3" s="3"/>
       <c r="I3" s="3"/>
       <c r="J3" s="3"/>
       <c r="K3" s="3"/>
     </row>
-    <row r="4" ht="22" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
-      <c r="J4" s="2"/>
-      <c r="K4" s="2"/>
-    </row>
-    <row r="5" ht="22" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" s="2"/>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
       <c r="H5" s="3"/>
       <c r="I5" s="3"/>
       <c r="J5" s="3"/>
       <c r="K5" s="3"/>
     </row>
-    <row r="6" ht="22" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="2"/>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
-      <c r="I6" s="2"/>
-      <c r="J6" s="2"/>
-      <c r="K6" s="2"/>
-    </row>
-    <row r="7" ht="22" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
+      <c r="J6" s="3"/>
+      <c r="K6" s="3"/>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" s="2"/>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
       <c r="H7" s="3"/>
       <c r="I7" s="3"/>
       <c r="J7" s="3"/>
       <c r="K7" s="3"/>
     </row>
-    <row r="8" ht="22" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="2"/>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
-      <c r="I8" s="2"/>
-      <c r="J8" s="2"/>
-      <c r="K8" s="2"/>
-    </row>
-    <row r="10" ht="28" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A10" s="4" t="s">
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
+      <c r="J8" s="3"/>
+      <c r="K8" s="3"/>
+    </row>
+    <row r="10" ht="26" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A10" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="B10" s="4"/>
-      <c r="C10" s="4"/>
-      <c r="D10" s="4"/>
-      <c r="E10" s="4"/>
-      <c r="F10" s="4"/>
-      <c r="G10" s="4"/>
-      <c r="H10" s="4"/>
-      <c r="I10" s="4"/>
-      <c r="J10" s="4"/>
-      <c r="K10" s="4"/>
-    </row>
-    <row r="11" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A11" s="5" t="s">
+      <c r="B10" s="6"/>
+      <c r="C10" s="6"/>
+      <c r="D10" s="6"/>
+      <c r="E10" s="6"/>
+      <c r="F10" s="6"/>
+      <c r="G10" s="6"/>
+      <c r="H10" s="6"/>
+      <c r="I10" s="6"/>
+      <c r="J10" s="6"/>
+      <c r="K10" s="6"/>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A11" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="B11" s="5"/>
-      <c r="C11" s="5"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
-      <c r="F11" s="5"/>
-      <c r="G11" s="5"/>
-      <c r="H11" s="5"/>
-      <c r="I11" s="5"/>
-      <c r="J11" s="5"/>
-      <c r="K11" s="5"/>
-    </row>
-    <row r="12" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A12" s="5" t="s">
+      <c r="B11" s="7"/>
+      <c r="C11" s="7"/>
+      <c r="D11" s="7"/>
+      <c r="E11" s="7"/>
+      <c r="F11" s="7"/>
+      <c r="G11" s="7"/>
+      <c r="H11" s="7"/>
+      <c r="I11" s="7"/>
+      <c r="J11" s="7"/>
+      <c r="K11" s="7"/>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A12" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="B12" s="5"/>
-      <c r="C12" s="5"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
-      <c r="F12" s="5"/>
-      <c r="G12" s="5"/>
-      <c r="H12" s="5"/>
-      <c r="I12" s="5"/>
-      <c r="J12" s="5"/>
-      <c r="K12" s="5"/>
-    </row>
-    <row r="13" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A13" s="5" t="s">
+      <c r="B12" s="7"/>
+      <c r="C12" s="7"/>
+      <c r="D12" s="7"/>
+      <c r="E12" s="7"/>
+      <c r="F12" s="7"/>
+      <c r="G12" s="7"/>
+      <c r="H12" s="7"/>
+      <c r="I12" s="7"/>
+      <c r="J12" s="7"/>
+      <c r="K12" s="7"/>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A13" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="B13" s="5"/>
-      <c r="C13" s="5"/>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
-      <c r="F13" s="5"/>
-      <c r="G13" s="5"/>
-      <c r="H13" s="5"/>
-      <c r="I13" s="5"/>
-      <c r="J13" s="5"/>
-      <c r="K13" s="5"/>
-    </row>
-    <row r="14" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A14" s="5" t="s">
+      <c r="B13" s="7"/>
+      <c r="C13" s="7"/>
+      <c r="D13" s="7"/>
+      <c r="E13" s="7"/>
+      <c r="F13" s="7"/>
+      <c r="G13" s="7"/>
+      <c r="H13" s="7"/>
+      <c r="I13" s="7"/>
+      <c r="J13" s="7"/>
+      <c r="K13" s="7"/>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A14" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="B14" s="5"/>
-      <c r="C14" s="5"/>
-      <c r="D14" s="5"/>
-      <c r="E14" s="5"/>
-      <c r="F14" s="5"/>
-      <c r="G14" s="5"/>
-      <c r="H14" s="5"/>
-      <c r="I14" s="5"/>
-      <c r="J14" s="5"/>
-      <c r="K14" s="5"/>
-    </row>
-    <row r="15" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A15" s="5" t="s">
+      <c r="B14" s="7"/>
+      <c r="C14" s="7"/>
+      <c r="D14" s="7"/>
+      <c r="E14" s="7"/>
+      <c r="F14" s="7"/>
+      <c r="G14" s="7"/>
+      <c r="H14" s="7"/>
+      <c r="I14" s="7"/>
+      <c r="J14" s="7"/>
+      <c r="K14" s="7"/>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A15" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="B15" s="5"/>
-      <c r="C15" s="5"/>
-      <c r="D15" s="5"/>
-      <c r="E15" s="5"/>
-      <c r="F15" s="5"/>
-      <c r="G15" s="5"/>
-      <c r="H15" s="5"/>
-      <c r="I15" s="5"/>
-      <c r="J15" s="5"/>
-      <c r="K15" s="5"/>
+      <c r="B15" s="7"/>
+      <c r="C15" s="7"/>
+      <c r="D15" s="7"/>
+      <c r="E15" s="7"/>
+      <c r="F15" s="7"/>
+      <c r="G15" s="7"/>
+      <c r="H15" s="7"/>
+      <c r="I15" s="7"/>
+      <c r="J15" s="7"/>
+      <c r="K15" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -2183,9 +2166,6 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr>
-    <tabColor rgb="1A1F2E"/>
-  </sheetPr>
   <dimension ref="A1:F20"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
@@ -2193,11 +2173,11 @@
     <col min="2" max="2" width="40" customWidth="1"/>
     <col min="3" max="3" width="55" customWidth="1"/>
     <col min="4" max="4" width="28" customWidth="1"/>
-    <col min="5" max="5" width="14" customWidth="1"/>
+    <col min="5" max="5" width="16" customWidth="1"/>
     <col min="6" max="6" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>77</v>
       </c>
@@ -2217,23 +2197,23 @@
         <v>82</v>
       </c>
     </row>
-    <row r="2" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="6"/>
-      <c r="B2" s="6"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
-      <c r="F2" s="6"/>
-    </row>
-    <row r="3" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="6"/>
-      <c r="B3" s="6"/>
-      <c r="C3" s="6"/>
-      <c r="D3" s="6"/>
-      <c r="E3" s="6"/>
-      <c r="F3" s="6"/>
-    </row>
-    <row r="4" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="8"/>
+      <c r="B2" s="8"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="8"/>
+      <c r="B3" s="8"/>
+      <c r="C3" s="8"/>
+      <c r="D3" s="8"/>
+      <c r="E3" s="8"/>
+      <c r="F3" s="8"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -2241,15 +2221,15 @@
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
     </row>
-    <row r="5" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-    </row>
-    <row r="6" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="2"/>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
@@ -2257,15 +2237,15 @@
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
     </row>
-    <row r="7" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="3"/>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-    </row>
-    <row r="8" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="2"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -2273,15 +2253,15 @@
       <c r="E8" s="2"/>
       <c r="F8" s="2"/>
     </row>
-    <row r="9" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="3"/>
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3"/>
-    </row>
-    <row r="10" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="2"/>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2"/>
+      <c r="F9" s="2"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -2289,15 +2269,15 @@
       <c r="E10" s="2"/>
       <c r="F10" s="2"/>
     </row>
-    <row r="11" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="3"/>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
-      <c r="F11" s="3"/>
-    </row>
-    <row r="12" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="2"/>
+      <c r="B11" s="2"/>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2"/>
+      <c r="F11" s="2"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
@@ -2305,75 +2285,75 @@
       <c r="E12" s="2"/>
       <c r="F12" s="2"/>
     </row>
-    <row r="14" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="7" t="s">
+    <row r="14" ht="26" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="B14" s="7"/>
-      <c r="C14" s="7"/>
-      <c r="D14" s="7"/>
-      <c r="E14" s="7"/>
-      <c r="F14" s="7"/>
-    </row>
-    <row r="15" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="5" t="s">
+      <c r="B14" s="10"/>
+      <c r="C14" s="10"/>
+      <c r="D14" s="10"/>
+      <c r="E14" s="10"/>
+      <c r="F14" s="10"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="B15" s="5"/>
-      <c r="C15" s="5"/>
-      <c r="D15" s="5"/>
-      <c r="E15" s="5"/>
-      <c r="F15" s="5"/>
-    </row>
-    <row r="16" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="5" t="s">
+      <c r="B15" s="7"/>
+      <c r="C15" s="7"/>
+      <c r="D15" s="7"/>
+      <c r="E15" s="7"/>
+      <c r="F15" s="7"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="B16" s="5"/>
-      <c r="C16" s="5"/>
-      <c r="D16" s="5"/>
-      <c r="E16" s="5"/>
-      <c r="F16" s="5"/>
-    </row>
-    <row r="17" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="5" t="s">
+      <c r="B16" s="7"/>
+      <c r="C16" s="7"/>
+      <c r="D16" s="7"/>
+      <c r="E16" s="7"/>
+      <c r="F16" s="7"/>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="B17" s="5"/>
-      <c r="C17" s="5"/>
-      <c r="D17" s="5"/>
-      <c r="E17" s="5"/>
-      <c r="F17" s="5"/>
-    </row>
-    <row r="18" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" s="5" t="s">
+      <c r="B17" s="7"/>
+      <c r="C17" s="7"/>
+      <c r="D17" s="7"/>
+      <c r="E17" s="7"/>
+      <c r="F17" s="7"/>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="B18" s="5"/>
-      <c r="C18" s="5"/>
-      <c r="D18" s="5"/>
-      <c r="E18" s="5"/>
-      <c r="F18" s="5"/>
-    </row>
-    <row r="19" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" s="5" t="s">
+      <c r="B18" s="7"/>
+      <c r="C18" s="7"/>
+      <c r="D18" s="7"/>
+      <c r="E18" s="7"/>
+      <c r="F18" s="7"/>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="B19" s="5"/>
-      <c r="C19" s="5"/>
-      <c r="D19" s="5"/>
-      <c r="E19" s="5"/>
-      <c r="F19" s="5"/>
-    </row>
-    <row r="20" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20" s="5" t="s">
+      <c r="B19" s="7"/>
+      <c r="C19" s="7"/>
+      <c r="D19" s="7"/>
+      <c r="E19" s="7"/>
+      <c r="F19" s="7"/>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="B20" s="5"/>
-      <c r="C20" s="5"/>
-      <c r="D20" s="5"/>
-      <c r="E20" s="5"/>
-      <c r="F20" s="5"/>
+      <c r="B20" s="7"/>
+      <c r="C20" s="7"/>
+      <c r="D20" s="7"/>
+      <c r="E20" s="7"/>
+      <c r="F20" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -2392,9 +2372,6 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr>
-    <tabColor rgb="1A1F2E"/>
-  </sheetPr>
   <dimension ref="A1:I20"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
@@ -2405,7 +2382,7 @@
     <col min="8" max="9" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>90</v>
       </c>
@@ -2434,134 +2411,134 @@
         <v>93</v>
       </c>
     </row>
-    <row r="2" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-    </row>
-    <row r="3" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
       <c r="G3" s="3"/>
       <c r="H3" s="3"/>
       <c r="I3" s="3"/>
     </row>
-    <row r="4" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
-    </row>
-    <row r="5" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" s="2"/>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
       <c r="G5" s="3"/>
       <c r="H5" s="3"/>
       <c r="I5" s="3"/>
     </row>
-    <row r="6" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
-      <c r="I6" s="2"/>
-    </row>
-    <row r="7" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="3"/>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" s="2"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
       <c r="G7" s="3"/>
       <c r="H7" s="3"/>
       <c r="I7" s="3"/>
     </row>
-    <row r="8" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
       <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
-      <c r="I8" s="2"/>
-    </row>
-    <row r="9" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="3"/>
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" s="2"/>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2"/>
+      <c r="F9" s="2"/>
       <c r="G9" s="3"/>
       <c r="H9" s="3"/>
       <c r="I9" s="3"/>
     </row>
-    <row r="10" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
       <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
-      <c r="H10" s="2"/>
-      <c r="I10" s="2"/>
-    </row>
-    <row r="11" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" s="3"/>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
-      <c r="F11" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+      <c r="I10" s="3"/>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" s="2"/>
+      <c r="B11" s="2"/>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2"/>
+      <c r="F11" s="2"/>
       <c r="G11" s="3"/>
       <c r="H11" s="3"/>
       <c r="I11" s="3"/>
     </row>
-    <row r="12" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
       <c r="F12" s="2"/>
-      <c r="G12" s="2"/>
-      <c r="H12" s="2"/>
-      <c r="I12" s="2"/>
-    </row>
-    <row r="13" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" s="3"/>
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3"/>
-      <c r="F13" s="3"/>
+      <c r="G12" s="3"/>
+      <c r="H12" s="3"/>
+      <c r="I12" s="3"/>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" s="2"/>
+      <c r="B13" s="2"/>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2"/>
+      <c r="F13" s="2"/>
       <c r="G13" s="3"/>
       <c r="H13" s="3"/>
       <c r="I13" s="3"/>
@@ -2573,43 +2550,43 @@
       <c r="D14" s="4"/>
       <c r="E14" s="4"/>
       <c r="F14" s="4"/>
-      <c r="G14" s="4"/>
-      <c r="H14" s="4"/>
-      <c r="I14" s="4"/>
-    </row>
-    <row r="16" ht="28" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A16" s="8" t="s">
+      <c r="G14" s="5"/>
+      <c r="H14" s="5"/>
+      <c r="I14" s="5"/>
+    </row>
+    <row r="16" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" s="11" t="s">
         <v>94</v>
       </c>
-      <c r="B16" s="8"/>
-      <c r="C16" s="8"/>
-      <c r="D16" s="8"/>
-      <c r="E16" s="8"/>
-      <c r="F16" s="8"/>
-      <c r="G16" s="8"/>
-      <c r="H16" s="8"/>
-      <c r="I16" s="8"/>
-    </row>
-    <row r="17" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A17" s="2"/>
-      <c r="B17" s="2"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
-      <c r="F17" s="2"/>
-      <c r="G17" s="2"/>
-      <c r="H17" s="2"/>
-      <c r="I17" s="2"/>
-    </row>
-    <row r="18" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A18" s="3"/>
-      <c r="B18" s="3"/>
-      <c r="C18" s="3"/>
-      <c r="D18" s="3"/>
-      <c r="E18" s="3"/>
-      <c r="F18" s="3"/>
-      <c r="G18" s="3"/>
-      <c r="H18" s="3"/>
+      <c r="B16" s="11"/>
+      <c r="C16" s="11"/>
+      <c r="D16" s="11"/>
+      <c r="E16" s="11"/>
+      <c r="F16" s="11"/>
+      <c r="G16" s="11"/>
+      <c r="H16" s="11"/>
+      <c r="I16" s="11"/>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A17" s="8"/>
+      <c r="B17" s="8"/>
+      <c r="C17" s="8"/>
+      <c r="D17" s="8"/>
+      <c r="E17" s="8"/>
+      <c r="F17" s="8"/>
+      <c r="G17" s="8"/>
+      <c r="H17" s="8"/>
+      <c r="I17" s="9"/>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" s="2"/>
+      <c r="B18" s="2"/>
+      <c r="C18" s="2"/>
+      <c r="D18" s="2"/>
+      <c r="E18" s="2"/>
+      <c r="F18" s="2"/>
+      <c r="G18" s="2"/>
+      <c r="H18" s="2"/>
       <c r="I18" s="3"/>
     </row>
     <row r="19" ht="26" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -2621,10 +2598,10 @@
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
-      <c r="I19" s="4"/>
+      <c r="I19" s="5"/>
     </row>
     <row r="20" spans="9:9" x14ac:dyDescent="0.25">
-      <c r="I20" s="9"/>
+      <c r="I20" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2637,10 +2614,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr>
-    <tabColor rgb="1A1F2E"/>
-  </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
@@ -2650,232 +2624,241 @@
     <col min="7" max="7" width="55" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="10" t="s">
+    <row r="1" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="13" t="s">
         <v>95</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10"/>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+    </row>
+    <row r="2" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" s="1" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="3" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="11"/>
-      <c r="B3" s="11"/>
-      <c r="C3" s="11"/>
-      <c r="D3" s="11"/>
-      <c r="E3" s="11"/>
-      <c r="F3" s="11"/>
-      <c r="G3" s="11"/>
-    </row>
-    <row r="4" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="3"/>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="2"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="2"/>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
       <c r="E4" s="3"/>
       <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
-    </row>
-    <row r="5" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G4" s="2"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="3"/>
-      <c r="B6" s="3"/>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="2"/>
+      <c r="B6" s="2"/>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
-      <c r="G6" s="3"/>
-    </row>
-    <row r="7" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G6" s="2"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
       <c r="G7" s="2"/>
     </row>
-    <row r="8" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="3"/>
-      <c r="B8" s="3"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="2"/>
+      <c r="B8" s="2"/>
+      <c r="C8" s="2"/>
+      <c r="D8" s="2"/>
       <c r="E8" s="3"/>
       <c r="F8" s="3"/>
-      <c r="G8" s="3"/>
-    </row>
-    <row r="11" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="12"/>
-      <c r="B11" s="12"/>
-      <c r="C11" s="12"/>
-      <c r="D11" s="12"/>
-      <c r="E11" s="12"/>
-      <c r="F11" s="12"/>
-      <c r="G11" s="12"/>
-    </row>
-    <row r="12" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="13"/>
-      <c r="B12" s="13"/>
-      <c r="C12" s="13"/>
-      <c r="D12" s="13"/>
-      <c r="E12" s="13"/>
-      <c r="F12" s="13"/>
-      <c r="G12" s="13"/>
-    </row>
-    <row r="13" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="4" t="s">
+      <c r="G8" s="2"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="8"/>
+      <c r="B10" s="8"/>
+      <c r="C10" s="8"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="9"/>
+      <c r="G10" s="8"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="4"/>
+      <c r="B11" s="4"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+      <c r="F11" s="3"/>
+      <c r="G11" s="4"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="4"/>
+      <c r="B12" s="4"/>
+      <c r="C12" s="4"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4"/>
+      <c r="F12" s="3"/>
+      <c r="G12" s="4"/>
+    </row>
+    <row r="14" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="B13" s="4"/>
-      <c r="C13" s="4"/>
-      <c r="D13" s="4"/>
-      <c r="E13" s="4"/>
-      <c r="F13" s="4"/>
-      <c r="G13" s="4"/>
-    </row>
-    <row r="14" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="2"/>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
-      <c r="G14" s="2"/>
-    </row>
-    <row r="15" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="3"/>
-      <c r="B15" s="3"/>
-      <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
+      <c r="B14" s="6"/>
+      <c r="C14" s="6"/>
+      <c r="D14" s="6"/>
+      <c r="E14" s="6"/>
+      <c r="F14" s="6"/>
+      <c r="G14" s="6"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" s="2"/>
+      <c r="B15" s="2"/>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
       <c r="E15" s="3"/>
       <c r="F15" s="3"/>
-      <c r="G15" s="3"/>
-    </row>
-    <row r="16" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G15" s="2"/>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
       <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
+      <c r="E16" s="3"/>
+      <c r="F16" s="3"/>
       <c r="G16" s="2"/>
     </row>
-    <row r="17" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="3"/>
-      <c r="B17" s="3"/>
-      <c r="C17" s="3"/>
-      <c r="D17" s="3"/>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" s="2"/>
+      <c r="B17" s="2"/>
+      <c r="C17" s="2"/>
+      <c r="D17" s="2"/>
       <c r="E17" s="3"/>
       <c r="F17" s="3"/>
-      <c r="G17" s="3"/>
-    </row>
-    <row r="18" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G17" s="2"/>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="2"/>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
       <c r="G18" s="2"/>
     </row>
-    <row r="20" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="7" t="s">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="2"/>
+      <c r="B19" s="2"/>
+      <c r="C19" s="2"/>
+      <c r="D19" s="2"/>
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
+      <c r="G19" s="2"/>
+    </row>
+    <row r="21" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="10" t="s">
         <v>104</v>
       </c>
-      <c r="B20" s="7"/>
-      <c r="C20" s="7"/>
-      <c r="D20" s="7"/>
-      <c r="E20" s="7"/>
-      <c r="F20" s="7"/>
-      <c r="G20" s="7"/>
-    </row>
-    <row r="21" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21" s="5" t="s">
+      <c r="B21" s="10"/>
+      <c r="C21" s="10"/>
+      <c r="D21" s="10"/>
+      <c r="E21" s="10"/>
+      <c r="F21" s="10"/>
+      <c r="G21" s="10"/>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="B21" s="5"/>
-      <c r="C21" s="5"/>
-      <c r="D21" s="5"/>
-      <c r="E21" s="5"/>
-      <c r="F21" s="5"/>
-      <c r="G21" s="5"/>
-    </row>
-    <row r="22" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="5" t="s">
+      <c r="B22" s="7"/>
+      <c r="C22" s="7"/>
+      <c r="D22" s="7"/>
+      <c r="E22" s="7"/>
+      <c r="F22" s="7"/>
+      <c r="G22" s="7"/>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="B22" s="5"/>
-      <c r="C22" s="5"/>
-      <c r="D22" s="5"/>
-      <c r="E22" s="5"/>
-      <c r="F22" s="5"/>
-      <c r="G22" s="5"/>
-    </row>
-    <row r="23" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="5" t="s">
+      <c r="B23" s="7"/>
+      <c r="C23" s="7"/>
+      <c r="D23" s="7"/>
+      <c r="E23" s="7"/>
+      <c r="F23" s="7"/>
+      <c r="G23" s="7"/>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="B23" s="5"/>
-      <c r="C23" s="5"/>
-      <c r="D23" s="5"/>
-      <c r="E23" s="5"/>
-      <c r="F23" s="5"/>
-      <c r="G23" s="5"/>
-    </row>
-    <row r="24" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="5" t="s">
+      <c r="B24" s="7"/>
+      <c r="C24" s="7"/>
+      <c r="D24" s="7"/>
+      <c r="E24" s="7"/>
+      <c r="F24" s="7"/>
+      <c r="G24" s="7"/>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="B24" s="5"/>
-      <c r="C24" s="5"/>
-      <c r="D24" s="5"/>
-      <c r="E24" s="5"/>
-      <c r="F24" s="5"/>
-      <c r="G24" s="5"/>
+      <c r="B25" s="7"/>
+      <c r="C25" s="7"/>
+      <c r="D25" s="7"/>
+      <c r="E25" s="7"/>
+      <c r="F25" s="7"/>
+      <c r="G25" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A13:G13"/>
-    <mergeCell ref="A20:G20"/>
+    <mergeCell ref="A14:G14"/>
     <mergeCell ref="A21:G21"/>
     <mergeCell ref="A22:G22"/>
     <mergeCell ref="A23:G23"/>
     <mergeCell ref="A24:G24"/>
+    <mergeCell ref="A25:G25"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>